<commit_message>
v5 - Positionsfix Teambuilder
</commit_message>
<xml_diff>
--- a/rollen_definitionen.xlsx
+++ b/rollen_definitionen.xlsx
@@ -2,10 +2,10 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rf4903cc497134dbb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rollen" sheetId="2" r:id="Re4afecd0bce94d00"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metriken" sheetId="3" r:id="R63eec8c37af240fc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source_Roles" sheetId="4" r:id="R5541b4d85c8b4c23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R13f458d3116843c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Rollen" sheetId="2" r:id="R5ed0780a8732407c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Metriken" sheetId="3" r:id="Rda9e2bf6fd2d4313"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source_Roles" sheetId="4" r:id="R80773c4033e44536"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -428,10 +428,8 @@
           <x:t xml:space="preserve">Änderungen 2026-05-17</x:t>
         </x:is>
       </x:c>
-      <x:c r="B6" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Mitspielender IV wurde in Aufbau-IV und Progressiver IV aufgeteilt; Klassische 10 und Kreativer Freigeist wurden zu Offensiver Kreativspieler zusammengeführt; Mittelfeld-/Offensivpositionsfamilien wurden vereinfacht.</x:t>
-        </x:is>
+      <x:c r="B6" s="3" t="str">
+        <x:v>IV-Rollen wurden in defensiv, Aufbau und progressiv aufgefächert; die offensiven Kreativrollen wurden zusammengeführt; Mittelfeld-/Offensivpositionsfamilien wurden vereinfacht.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -607,10 +605,8 @@
       <x:c r="D5" s="3" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E5" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Ersetzt einen Teil der bisherigen Rolle Mitspielender IV.</x:t>
-        </x:is>
+      <x:c r="E5" s="3" t="str">
+        <x:v>Neue IV-Aufteilung: aufbauorientiertes Innenverteidigerprofil.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
@@ -632,10 +628,8 @@
       <x:c r="D6" s="3" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E6" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Ersetzt einen Teil der bisherigen Rolle Mitspielender IV.</x:t>
-        </x:is>
+      <x:c r="E6" s="3" t="str">
+        <x:v>Neue IV-Aufteilung: progressives Innenverteidigerprofil.</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
@@ -805,10 +799,8 @@
       <x:c r="D13" s="3" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="E13" s="3" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">Zusammenführung aus Klassische 10 und Kreativer Freigeist.</x:t>
-        </x:is>
+      <x:c r="E13" s="3" t="str">
+        <x:v>Zusammengeführtes offensives Kreativprofil.</x:v>
       </x:c>
     </x:row>
     <x:row r="14">

</xml_diff>